<commit_message>
Fix template row-wiring, 32,767 wording, moonfish README clarity
</commit_message>
<xml_diff>
--- a/GenBank_Annotation_Template.xlsx
+++ b/GenBank_Annotation_Template.xlsx
@@ -653,7 +653,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>The nucleotide sequence itself goes on the separate "Sequence" sheet, not here — Excel caps a single cell at about 32,000 characters, which most real genomes exceed, so that sheet lets you split the sequence across multiple cells. Required — used to sanity-check feature coordinates and (for the .gb output) to compute CDS translations.</t>
+          <t>The nucleotide sequence itself goes on the separate "Sequence" sheet, not here — Excel caps a single cell at 32,767 characters (the actual Excel limit), which most real genomes exceed, so that sheet lets you split the sequence across multiple cells. Required — used to sanity-check feature coordinates and (for the .gb output) to compute CDS translations.</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1417,7 @@
     <row r="1" ht="60" customHeight="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>Paste your nucleotide sequence below, starting in cell A2 — one continuous string per cell, no spaces/numbers/line breaks (A/C/G/T/U and standard IUPAC ambiguity codes only). Excel limits a single cell to about 32,000 characters, so for anything longer than that (most real genomes), split the sequence across multiple cells in this column (A2, A3, A4, ...) IN ORDER — the scripts read down the column and join the cells together, so where you break the sequence between cells does not matter as long as the order is right. Don't put anything else on this sheet.</t>
+          <t>Paste your nucleotide sequence below, starting in cell A2 — one continuous string per cell, no spaces/numbers/line breaks (A/C/G/T/U and standard IUPAC ambiguity codes only). Excel limits a single cell to 32,767 characters (the actual Excel limit), so for anything longer than that (most real genomes), split the sequence across multiple cells in this column (A2, A3, A4, ...) IN ORDER — the scripts read down the column and join the cells together, so where you break the sequence between cells does not matter as long as the order is right. Don't put anything else on this sheet.</t>
         </is>
       </c>
     </row>

</xml_diff>